<commit_message>
NPB自動更新(2軍): 2026-09-22 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/2軍/公式戦/raw/2026-09-22/highlights_20260922.xlsx
+++ b/data/プロ野球/2026年/2軍/公式戦/raw/2026-09-22/highlights_20260922.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>10回裏にサヨナラタイムリーツーベースを放ち、延長戦に終止符を打った。</t>
+          <t>延長10回裏にサヨナラタイムリーツーベースを放ち、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -504,17 +504,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>田村 俊介</t>
+          <t>森 駿太</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>広島</t>
+          <t>中日</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7回裏に勝ち越しタイムリーツーベースを放ち、接戦を制する大きな一打となった。</t>
+          <t>8回表に同点タイムリーヒットを放ち、試合を振り出しに戻す活躍を見せた。</t>
         </is>
       </c>
     </row>
@@ -529,17 +529,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>柿沼 友哉</t>
+          <t>田村 俊介</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ヤクルト</t>
+          <t>広島</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8回裏に勝ち越し犠牲フライを放ち、チームを勝利に導く貴重な打点を挙げた。</t>
+          <t>7回裏に勝ち越しタイムリーツーベースを放ち、チームの勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -554,17 +554,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>森 駿太</t>
+          <t>柿沼 友哉</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>中日</t>
+          <t>ヤクルト</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>8回表に同点タイムリーヒットを放ち、土壇場で試合を振り出しに戻した。</t>
+          <t>8回裏に勝ち越し犠牲フライを放ち、接戦を制する貴重な打点を挙げた。</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6回裏に同点2ランホームランを放ち、試合の流れを大きく引き寄せた。</t>
+          <t>6回裏に同点2ランホームランを放ち、チームの反撃の狼煙を上げた。</t>
         </is>
       </c>
     </row>

</xml_diff>